<commit_message>
Torna a base autossuficiente e adiciona atualização incremental pelo podcast
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0193kkcaFr2zeWvcQdmPTqWt
</commit_message>
<xml_diff>
--- a/sermoes/sermoes_fdqc_completa.xlsx
+++ b/sermoes/sermoes_fdqc_completa.xlsx
@@ -24388,7 +24388,7 @@
       </c>
       <c r="N279" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-que-e-uma-igreja-parte-2-leandro-vieira-minisserie-igreja-o-evangelho-visivel</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-que-e-uma-igreja-leandro-vieira-minisserie-igreja-o-evangelho-visivel</t>
         </is>
       </c>
       <c r="O279" t="inlineStr">
@@ -33650,7 +33650,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>20/05/2019</t>
+          <t>23/05/2019</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
@@ -33663,37 +33663,42 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>Rápidos para Ouvir - Fabiano Krehnke</t>
+          <t>O Nosso Resgatador - Leandro Alves</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>Fabiano Krehnke</t>
+          <t>Leandro Alves</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Tg 1.19-27</t>
+          <t>Rt 1–4</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t>Tiago</t>
+          <t>Rute</t>
         </is>
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>Tg 1</t>
+          <t>Rt 1–4</t>
         </is>
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t>Novo Testamento</t>
+          <t>Antigo Testamento</t>
         </is>
       </c>
       <c r="J391" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
@@ -33703,39 +33708,44 @@
       </c>
       <c r="M391" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/lugar-de-fala-vs-lugar-de-escuta-fabiano-krehnke</t>
+          <t>https://www.youtube.com/watch?v=jFc2sOuPvys</t>
         </is>
       </c>
       <c r="N391" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/lugar-de-fala-vs-lugar-de-escuta-fabiano-krehnke</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-nosso-resgatador-leandro-alves</t>
         </is>
       </c>
       <c r="O391" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
       <c r="P391" t="inlineStr">
         <is>
-          <t>Transcrição do áudio</t>
+          <t>NotebookLM</t>
+        </is>
+      </c>
+      <c r="R391" t="inlineStr">
+        <is>
+          <t>Rute 1:1-21; 2:5-12; 3:9-12; 4:6-18</t>
         </is>
       </c>
       <c r="S391" t="inlineStr">
         <is>
-          <t>P193</t>
+          <t>Y164</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>17/05/2019</t>
+          <t>20/05/2019</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>12/05/2019</t>
+          <t>19/05/2019</t>
         </is>
       </c>
       <c r="C392" t="n">
@@ -33743,12 +33753,32 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Identidade, Natureza e Propósito - Paulo Borges Junior</t>
+          <t>Rápidos para Ouvir - Fabiano Krehnke</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>Paulo Borges Junior</t>
+          <t>Fabiano Krehnke</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Tg 1.19-27</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Tiago</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>Tg 1</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Novo Testamento</t>
         </is>
       </c>
       <c r="J392" t="inlineStr">
@@ -33763,29 +33793,34 @@
       </c>
       <c r="M392" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=OOcRJ22joWo</t>
+          <t>https://soundcloud.com/familiadosquecreem/lugar-de-fala-vs-lugar-de-escuta-fabiano-krehnke</t>
         </is>
       </c>
       <c r="N392" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-evangelho-da-igreja-paulo-borges-jr-com-todos-os-santos</t>
+          <t>https://soundcloud.com/familiadosquecreem/lugar-de-fala-vs-lugar-de-escuta-fabiano-krehnke</t>
         </is>
       </c>
       <c r="O392" t="inlineStr">
         <is>
-          <t>Temático</t>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="P392" t="inlineStr">
+        <is>
+          <t>Transcrição do áudio</t>
         </is>
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t>Y233</t>
+          <t>P193</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>15/05/2019</t>
+          <t>17/05/2019</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -33798,7 +33833,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Uns aos Outros - Paulo Borges Junior</t>
+          <t>Identidade, Natureza e Propósito - Paulo Borges Junior</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -33818,12 +33853,12 @@
       </c>
       <c r="M393" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=tpUb7nO-t6o</t>
+          <t>https://www.youtube.com/watch?v=OOcRJ22joWo</t>
         </is>
       </c>
       <c r="N393" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/uns-aos-outros-paulo-borges-jr-com-todos-os-santos</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-evangelho-da-igreja-paulo-borges-jr-com-todos-os-santos</t>
         </is>
       </c>
       <c r="O393" t="inlineStr">
@@ -33833,14 +33868,14 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t>Y234</t>
+          <t>Y233</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>13/05/2019</t>
+          <t>15/05/2019</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
@@ -33853,7 +33888,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>O Evangelho da Igreja - Paulo Borges Junior</t>
+          <t>Uns aos Outros - Paulo Borges Junior</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -33873,12 +33908,12 @@
       </c>
       <c r="M394" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Hw27wxncTvs</t>
+          <t>https://www.youtube.com/watch?v=tpUb7nO-t6o</t>
         </is>
       </c>
       <c r="N394" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/identidade-natureza-e-proposito-paulo-borges-jr-com-todos-os-santos</t>
+          <t>https://soundcloud.com/familiadosquecreem/uns-aos-outros-paulo-borges-jr-com-todos-os-santos</t>
         </is>
       </c>
       <c r="O394" t="inlineStr">
@@ -33888,19 +33923,19 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t>Y235</t>
+          <t>Y234</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>10/05/2019</t>
+          <t>13/05/2019</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>05/05/2019</t>
+          <t>12/05/2019</t>
         </is>
       </c>
       <c r="C395" t="n">
@@ -33908,32 +33943,12 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>O Poder da Ressurreição - Leandro Vieira</t>
+          <t>O Evangelho da Igreja - Paulo Borges Junior</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
-        </is>
-      </c>
-      <c r="F395" t="inlineStr">
-        <is>
-          <t>2Ts 3.6</t>
-        </is>
-      </c>
-      <c r="G395" t="inlineStr">
-        <is>
-          <t>2 Tessalonicenses</t>
-        </is>
-      </c>
-      <c r="H395" t="inlineStr">
-        <is>
-          <t>2Ts 3</t>
-        </is>
-      </c>
-      <c r="I395" t="inlineStr">
-        <is>
-          <t>Novo Testamento</t>
+          <t>Paulo Borges Junior</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
@@ -33948,34 +33963,29 @@
       </c>
       <c r="M395" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-poder-da-ressurreicao-leandro-vieira</t>
+          <t>https://www.youtube.com/watch?v=Hw27wxncTvs</t>
         </is>
       </c>
       <c r="N395" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-poder-da-ressurreicao-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/identidade-natureza-e-proposito-paulo-borges-jr-com-todos-os-santos</t>
         </is>
       </c>
       <c r="O395" t="inlineStr">
         <is>
-          <t>Provável</t>
-        </is>
-      </c>
-      <c r="P395" t="inlineStr">
-        <is>
-          <t>Transcrição do áudio</t>
+          <t>Temático</t>
         </is>
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t>P194</t>
+          <t>Y235</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>06/05/2019</t>
+          <t>10/05/2019</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
@@ -33988,7 +33998,7 @@
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>Valor de Uma História Profética - Leandro Vieira</t>
+          <t>O Poder da Ressurreição - Leandro Vieira</t>
         </is>
       </c>
       <c r="E396" t="inlineStr">
@@ -33998,22 +34008,22 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Sl 139.13-16</t>
+          <t>2Ts 3.6</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t>Salmos</t>
+          <t>2 Tessalonicenses</t>
         </is>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>Sl 139</t>
+          <t>2Ts 3</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>Antigo Testamento</t>
+          <t>Novo Testamento</t>
         </is>
       </c>
       <c r="J396" t="inlineStr">
@@ -34028,12 +34038,12 @@
       </c>
       <c r="M396" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/valor-de-uma-historia-profetica-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-poder-da-ressurreicao-leandro-vieira</t>
         </is>
       </c>
       <c r="N396" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/valor-de-uma-historia-profetica-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-poder-da-ressurreicao-leandro-vieira</t>
         </is>
       </c>
       <c r="O396" t="inlineStr">
@@ -34048,19 +34058,19 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t>P195</t>
+          <t>P194</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>24/04/2019</t>
+          <t>06/05/2019</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>21/04/2019</t>
+          <t>05/05/2019</t>
         </is>
       </c>
       <c r="C397" t="n">
@@ -34068,42 +34078,37 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 3) - Leandro Alves</t>
+          <t>Valor de Uma História Profética - Leandro Vieira</t>
         </is>
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>Mt 5.17-20?</t>
+          <t>Sl 139.13-16</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>Salmos</t>
         </is>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t>Mt 5</t>
+          <t>Sl 139</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>Novo Testamento</t>
+          <t>Antigo Testamento</t>
         </is>
       </c>
       <c r="J397" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K397" t="inlineStr">
-        <is>
-          <t>Fundamentos do NT</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
@@ -34113,49 +34118,39 @@
       </c>
       <c r="M397" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=6O7tAVbxCqA</t>
+          <t>https://soundcloud.com/familiadosquecreem/valor-de-uma-historia-profetica-leandro-vieira</t>
         </is>
       </c>
       <c r="N397" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-reino-parte-3-leandro-alves</t>
+          <t>https://soundcloud.com/familiadosquecreem/valor-de-uma-historia-profetica-leandro-vieira</t>
         </is>
       </c>
       <c r="O397" t="inlineStr">
         <is>
-          <t>Incerto</t>
+          <t>Provável</t>
         </is>
       </c>
       <c r="P397" t="inlineStr">
         <is>
-          <t>NotebookLM</t>
-        </is>
-      </c>
-      <c r="Q397" t="inlineStr">
-        <is>
-          <t>…esta ideia, com esse entendimento, e aí entramos o texto de Marcos, capítulo 1, onde o Leandro falou sobre a chegada do reino. Então se você quiser notar, estiver notando só para gente trazer uma introdução para aqueles que nã…</t>
-        </is>
-      </c>
-      <c r="R397" t="inlineStr">
-        <is>
-          <t>Mateus 5:1-48; Mateus 5:17-20; Hebreus 10:16 (o áudio do podcast cita Mc 1.15; Lc 11.20; 22.18)</t>
+          <t>Transcrição do áudio</t>
         </is>
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>P195</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>03/04/2019</t>
+          <t>24/04/2019</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>31/03/2019</t>
+          <t>21/04/2019</t>
         </is>
       </c>
       <c r="C398" t="n">
@@ -34163,17 +34158,17 @@
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 2) - Felipe Bartoszewski</t>
+          <t>Fundamentos: Reino (parte 3) - Leandro Alves</t>
         </is>
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Felipe Bartoszewski</t>
+          <t>Leandro Alves</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Mt 16.13-28</t>
+          <t>Mt 5.17-20?</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -34183,7 +34178,7 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t>Mt 16</t>
+          <t>Mt 5</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
@@ -34208,49 +34203,49 @@
       </c>
       <c r="M398" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=sYDC9JZC7xU</t>
+          <t>https://www.youtube.com/watch?v=6O7tAVbxCqA</t>
         </is>
       </c>
       <c r="N398" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-reino-parte-2-felipe-bartoszewski</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-reino-parte-3-leandro-alves</t>
         </is>
       </c>
       <c r="O398" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Incerto</t>
         </is>
       </c>
       <c r="P398" t="inlineStr">
         <is>
-          <t>Transcrição + NotebookLM</t>
+          <t>NotebookLM</t>
         </is>
       </c>
       <c r="Q398" t="inlineStr">
         <is>
-          <t>…ntos, gente. Então, vamos falar sobre o contexto geral, né? Mateus, capítulo 16, Jesus está falando sobre a edificação da igreja. Ele está lançando os quatro fundamentos pelo qual o novo testamento ele está alicersado. Então,…</t>
+          <t>…esta ideia, com esse entendimento, e aí entramos o texto de Marcos, capítulo 1, onde o Leandro falou sobre a chegada do reino. Então se você quiser notar, estiver notando só para gente trazer uma introdução para aqueles que nã…</t>
         </is>
       </c>
       <c r="R398" t="inlineStr">
         <is>
-          <t>Mateus 16:13-28; Romanos 14:17; Gênesis 3</t>
+          <t>Mateus 5:1-48; Mateus 5:17-20; Hebreus 10:16 (o áudio do podcast cita Mc 1.15; Lc 11.20; 22.18)</t>
         </is>
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t>Y162</t>
+          <t>Y163</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>29/03/2019</t>
+          <t>03/04/2019</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>24/03/2019</t>
+          <t>31/03/2019</t>
         </is>
       </c>
       <c r="C399" t="n">
@@ -34258,27 +34253,27 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 1) - Leandro Vieira</t>
+          <t>Fundamentos: Reino (parte 2) - Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Mc 1.15; Lc 11.20</t>
+          <t>Mt 16.13-28</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t>Marcos, Lucas</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>Mc 1; Lc 11</t>
+          <t>Mt 16</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
@@ -34303,12 +34298,12 @@
       </c>
       <c r="M399" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TaBRibliwSE</t>
+          <t>https://www.youtube.com/watch?v=sYDC9JZC7xU</t>
         </is>
       </c>
       <c r="N399" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-reino-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-reino-parte-2-felipe-bartoszewski</t>
         </is>
       </c>
       <c r="O399" t="inlineStr">
@@ -34323,29 +34318,29 @@
       </c>
       <c r="Q399" t="inlineStr">
         <is>
-          <t>…. Então, precha atenção. No início do Ministério do Cristo, marcos capitulo 1, verso 15, o Senhor disse, o tempo foi comprido e o reino de Deus está próximo a rependeivos e crede no Evangelho. Qual é a primeira evidência do re…</t>
+          <t>…ntos, gente. Então, vamos falar sobre o contexto geral, né? Mateus, capítulo 16, Jesus está falando sobre a edificação da igreja. Ele está lançando os quatro fundamentos pelo qual o novo testamento ele está alicersado. Então,…</t>
         </is>
       </c>
       <c r="R399" t="inlineStr">
         <is>
-          <t>Marcos 1:15; Lucas 11:20; Marcos 10:29-30</t>
+          <t>Mateus 16:13-28; Romanos 14:17; Gênesis 3</t>
         </is>
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t>Y161</t>
+          <t>Y162</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>22/03/2019</t>
+          <t>29/03/2019</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>17/03/2019</t>
+          <t>24/03/2019</t>
         </is>
       </c>
       <c r="C400" t="n">
@@ -34353,7 +34348,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>Fundamentos: Cruz (parte 02) - Leandro Vieira</t>
+          <t>Fundamentos: Reino (parte 1) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
@@ -34363,17 +34358,17 @@
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Gl 3.1</t>
+          <t>Mc 1.15; Lc 11.20</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t>Gálatas</t>
+          <t>Marcos, Lucas</t>
         </is>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>Gl 3</t>
+          <t>Mc 1; Lc 11</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
@@ -34398,12 +34393,12 @@
       </c>
       <c r="M400" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=2G_aK81vYpo</t>
+          <t>https://www.youtube.com/watch?v=TaBRibliwSE</t>
         </is>
       </c>
       <c r="N400" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-cruz-parte-02-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-reino-leandro-vieira</t>
         </is>
       </c>
       <c r="O400" t="inlineStr">
@@ -34413,24 +34408,29 @@
       </c>
       <c r="P400" t="inlineStr">
         <is>
-          <t>Transcrição do áudio</t>
+          <t>Transcrição + NotebookLM</t>
         </is>
       </c>
       <c r="Q400" t="inlineStr">
         <is>
-          <t>…s que é a cruz, e uma coisa que eu quero de novo ressaltar, Galatas Capítulo 3, por favor, versículo 1. Corre um pouquinho mais hoje, irmão. Galatas Capítulo 3, verso 1, nós abordamos esse texto na semana passada, já é uma das…</t>
+          <t>…. Então, precha atenção. No início do Ministério do Cristo, marcos capitulo 1, verso 15, o Senhor disse, o tempo foi comprido e o reino de Deus está próximo a rependeivos e crede no Evangelho. Qual é a primeira evidência do re…</t>
+        </is>
+      </c>
+      <c r="R400" t="inlineStr">
+        <is>
+          <t>Marcos 1:15; Lucas 11:20; Marcos 10:29-30</t>
         </is>
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t>Y160</t>
+          <t>Y161</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>18/03/2019</t>
+          <t>22/03/2019</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
@@ -34443,7 +34443,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Fundamentos: Cruz (parte 01) - Leandro Vieira</t>
+          <t>Fundamentos: Cruz (parte 02) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
@@ -34453,17 +34453,17 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>1Co 1.23</t>
+          <t>Gl 3.1</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
         <is>
-          <t>1 Coríntios</t>
+          <t>Gálatas</t>
         </is>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>1Co 1</t>
+          <t>Gl 3</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
@@ -34488,12 +34488,12 @@
       </c>
       <c r="M401" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=00rx_NzGu70</t>
+          <t>https://www.youtube.com/watch?v=2G_aK81vYpo</t>
         </is>
       </c>
       <c r="N401" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-cruz-parte-01-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-cruz-parte-02-leandro-vieira</t>
         </is>
       </c>
       <c r="O401" t="inlineStr">
@@ -34508,24 +34508,24 @@
       </c>
       <c r="Q401" t="inlineStr">
         <is>
-          <t>…reciso de tempo hoje. E eu quero que comecemos por primeira corinte os capítulos 1, versículo 23. Essa é das antiga. Essa é das antiga. Se não for, não dá, não. Eu queria tanto cantar, irmão. Consigo, irmão. Consigo, irmão. E…</t>
+          <t>…s que é a cruz, e uma coisa que eu quero de novo ressaltar, Galatas Capítulo 3, por favor, versículo 1. Corre um pouquinho mais hoje, irmão. Galatas Capítulo 3, verso 1, nós abordamos esse texto na semana passada, já é uma das…</t>
         </is>
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t>Y159</t>
+          <t>Y160</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>11/03/2019</t>
+          <t>18/03/2019</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>10/03/2019</t>
+          <t>17/03/2019</t>
         </is>
       </c>
       <c r="C402" t="n">
@@ -34533,27 +34533,27 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Fundamentos: Igreja - Leandro Alves</t>
+          <t>Fundamentos: Cruz (parte 01) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t>Mt 16.13-18</t>
+          <t>1Co 1.23</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>1 Coríntios</t>
         </is>
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t>Mt 16</t>
+          <t>1Co 1</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
@@ -34578,12 +34578,12 @@
       </c>
       <c r="M402" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=-vmjd4zLRH4</t>
+          <t>https://www.youtube.com/watch?v=00rx_NzGu70</t>
         </is>
       </c>
       <c r="N402" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-igreja-leandro-alves</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-cruz-parte-01-leandro-vieira</t>
         </is>
       </c>
       <c r="O402" t="inlineStr">
@@ -34593,34 +34593,29 @@
       </c>
       <c r="P402" t="inlineStr">
         <is>
-          <t>Transcrição + NotebookLM</t>
+          <t>Transcrição do áudio</t>
         </is>
       </c>
       <c r="Q402" t="inlineStr">
         <is>
-          <t>…. Eu gostaria somente que você anotasse o texto de primeiro Corinthians, capítulo 3, verso 10 e 11, que fala sobre Cristo, sendo a licer-se e efésios dois-vinte, que traz Cristo como fundamento dos apóstolos e dos profetas, o…</t>
-        </is>
-      </c>
-      <c r="R402" t="inlineStr">
-        <is>
-          <t>Mateus 16:13-18; Hebreus 3:1-6; Atos 2:42</t>
+          <t>…reciso de tempo hoje. E eu quero que comecemos por primeira corinte os capítulos 1, versículo 23. Essa é das antiga. Essa é das antiga. Se não for, não dá, não. Eu queria tanto cantar, irmão. Consigo, irmão. Consigo, irmão. E…</t>
         </is>
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t>Y158</t>
+          <t>Y159</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>01/03/2019</t>
+          <t>11/03/2019</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>24/02/2019</t>
+          <t>10/03/2019</t>
         </is>
       </c>
       <c r="C403" t="n">
@@ -34628,29 +34623,29 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Fundamentos: Cristo (parte 02) - Leandro Vieira</t>
+          <t>Fundamentos: Igreja - Leandro Alves</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Leandro Alves</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
+          <t>Mt 16.13-18</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Mateus</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
           <t>Mt 16</t>
         </is>
       </c>
-      <c r="G403" t="inlineStr">
-        <is>
-          <t>Mateus</t>
-        </is>
-      </c>
-      <c r="H403" t="inlineStr">
-        <is>
-          <t>Mt 16</t>
-        </is>
-      </c>
       <c r="I403" t="inlineStr">
         <is>
           <t>Novo Testamento</t>
@@ -34673,12 +34668,12 @@
       </c>
       <c r="M403" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=XNM_xEO_eaM</t>
+          <t>https://www.youtube.com/watch?v=-vmjd4zLRH4</t>
         </is>
       </c>
       <c r="N403" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-cristo-parte-02-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-igreja-leandro-alves</t>
         </is>
       </c>
       <c r="O403" t="inlineStr">
@@ -34688,29 +34683,34 @@
       </c>
       <c r="P403" t="inlineStr">
         <is>
-          <t>Transcrição do áudio</t>
+          <t>Transcrição + NotebookLM</t>
         </is>
       </c>
       <c r="Q403" t="inlineStr">
         <is>
-          <t>…Pra que a gente possa começar da forma correta, vamos abrir Mateus Capítulo 16 e eu vou diretamente aos textos que falam a respeito desses quatro fundamentos e vamos compartilhar. Primeiro versículo, o 16, 16, 16, 2 evangelho…</t>
+          <t>…. Eu gostaria somente que você anotasse o texto de primeiro Corinthians, capítulo 3, verso 10 e 11, que fala sobre Cristo, sendo a licer-se e efésios dois-vinte, que traz Cristo como fundamento dos apóstolos e dos profetas, o…</t>
+        </is>
+      </c>
+      <c r="R403" t="inlineStr">
+        <is>
+          <t>Mateus 16:13-18; Hebreus 3:1-6; Atos 2:42</t>
         </is>
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t>Y157</t>
+          <t>Y158</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>19/02/2019</t>
+          <t>01/03/2019</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>17/02/2019</t>
+          <t>24/02/2019</t>
         </is>
       </c>
       <c r="C404" t="n">
@@ -34718,17 +34718,17 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>Fundamentos: Cristo (parte 01) - Fabiano Krehnke</t>
+          <t>Fundamentos: Cristo (parte 02) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>Fabiano Krehnke</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t>Mt 16.13-16</t>
+          <t>Mt 16</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -34763,12 +34763,12 @@
       </c>
       <c r="M404" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=0Qj2iO2fWR8</t>
+          <t>https://www.youtube.com/watch?v=XNM_xEO_eaM</t>
         </is>
       </c>
       <c r="N404" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/fundamentos-do-novo-testamento-fabiano-krehnke</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-cristo-parte-02-leandro-vieira</t>
         </is>
       </c>
       <c r="O404" t="inlineStr">
@@ -34783,24 +34783,24 @@
       </c>
       <c r="Q404" t="inlineStr">
         <is>
-          <t>…como Pedro fala? Você, tu é o Cristo, o filho do Deus vivo, versículo 16, tu é o Cristo, o filho do Deus vivo, automaticamente assim que Pedro fala isso, Jesus vem e fala quem Ele é, percebe? Então Pedro recl...…</t>
+          <t>…Pra que a gente possa começar da forma correta, vamos abrir Mateus Capítulo 16 e eu vou diretamente aos textos que falam a respeito desses quatro fundamentos e vamos compartilhar. Primeiro versículo, o 16, 16, 16, 2 evangelho…</t>
         </is>
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t>Y156</t>
+          <t>Y157</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>16/02/2019</t>
+          <t>19/02/2019</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>10/02/2019</t>
+          <t>17/02/2019</t>
         </is>
       </c>
       <c r="C405" t="n">
@@ -34808,17 +34808,17 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Introdução aos Fundamentos do NT - Leandro Vieira</t>
+          <t>Fundamentos: Cristo (parte 01) - Fabiano Krehnke</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Fabiano Krehnke</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Mt 16.13-28</t>
+          <t>Mt 16.13-16</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -34853,12 +34853,12 @@
       </c>
       <c r="M405" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=X7jGPttaO5g</t>
+          <t>https://www.youtube.com/watch?v=0Qj2iO2fWR8</t>
         </is>
       </c>
       <c r="N405" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/introducao-aos-fundamentos-do-novo-testamento-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/fundamentos-do-novo-testamento-fabiano-krehnke</t>
         </is>
       </c>
       <c r="O405" t="inlineStr">
@@ -34873,24 +34873,24 @@
       </c>
       <c r="Q405" t="inlineStr">
         <is>
-          <t>…a que se abre esqueci disso então gente abre a escritura em Mateus capítulo 16 vamos ver do verso 13 vamos fazer uma leitura dinâmica e aí depois retornaremos aos pontos que eu desejo ressaltar o vanjel de Mateus capítulo 16 o…</t>
+          <t>…como Pedro fala? Você, tu é o Cristo, o filho do Deus vivo, versículo 16, tu é o Cristo, o filho do Deus vivo, automaticamente assim que Pedro fala isso, Jesus vem e fala quem Ele é, percebe? Então Pedro recl...…</t>
         </is>
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t>Y155</t>
+          <t>Y156</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>07/02/2019</t>
+          <t>16/02/2019</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>03/02/2019</t>
+          <t>10/02/2019</t>
         </is>
       </c>
       <c r="C406" t="n">
@@ -34898,27 +34898,27 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Batismo nas Águas, no Espírito e no Corpo - Felipe Bartoszewski</t>
+          <t>Introdução aos Fundamentos do NT - Leandro Vieira</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Felipe Bartoszewski</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>Hb 5–6</t>
+          <t>Mt 16.13-28</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
         <is>
-          <t>Hebreus</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>Hb 5–6</t>
+          <t>Mt 16</t>
         </is>
       </c>
       <c r="I406" t="inlineStr">
@@ -34928,7 +34928,12 @@
       </c>
       <c r="J406" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="L406" t="inlineStr">
@@ -34938,17 +34943,17 @@
       </c>
       <c r="M406" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/batismo-nas-aguas-no-espirito-e-no-corpo-felipe-bartoszewski</t>
+          <t>https://www.youtube.com/watch?v=X7jGPttaO5g</t>
         </is>
       </c>
       <c r="N406" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/batismo-nas-aguas-no-espirito-e-no-corpo-felipe-bartoszewski</t>
+          <t>https://soundcloud.com/familiadosquecreem/introducao-aos-fundamentos-do-novo-testamento-leandro-vieira</t>
         </is>
       </c>
       <c r="O406" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
       <c r="P406" t="inlineStr">
@@ -34956,16 +34961,21 @@
           <t>Transcrição do áudio</t>
         </is>
       </c>
+      <c r="Q406" t="inlineStr">
+        <is>
+          <t>…a que se abre esqueci disso então gente abre a escritura em Mateus capítulo 16 vamos ver do verso 13 vamos fazer uma leitura dinâmica e aí depois retornaremos aos pontos que eu desejo ressaltar o vanjel de Mateus capítulo 16 o…</t>
+        </is>
+      </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t>P196</t>
+          <t>Y155</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>04/02/2019</t>
+          <t>07/02/2019</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -34978,27 +34988,27 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>Série: Síndrome dos Gálatas (parte 3) - Leandro Vieira</t>
+          <t>Batismo nas Águas, no Espírito e no Corpo - Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Gl 1</t>
+          <t>Hb 5–6</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
         <is>
-          <t>Gálatas</t>
+          <t>Hebreus</t>
         </is>
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t>Gl 1</t>
+          <t>Hb 5–6</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
@@ -35008,12 +35018,7 @@
       </c>
       <c r="J407" t="inlineStr">
         <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="K407" t="inlineStr">
-        <is>
-          <t>Síndrome dos Gálatas</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
@@ -35023,12 +35028,12 @@
       </c>
       <c r="M407" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=qMRyQ6JDeZc</t>
+          <t>https://soundcloud.com/familiadosquecreem/batismo-nas-aguas-no-espirito-e-no-corpo-felipe-bartoszewski</t>
         </is>
       </c>
       <c r="N407" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/sindrome-dos-galatas-parte-03-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/batismo-nas-aguas-no-espirito-e-no-corpo-felipe-bartoszewski</t>
         </is>
       </c>
       <c r="O407" t="inlineStr">
@@ -35041,26 +35046,21 @@
           <t>Transcrição do áudio</t>
         </is>
       </c>
-      <c r="Q407" t="inlineStr">
-        <is>
-          <t>…m literatura. Amém? Por favor, irmão. Dedique tempo. Vamos agálatas. Capítulo 1. Galatas Capítulo 1, quem encontrou e diga assim. Então, qual é o tema da palavra, as síndromes dos galatas do Evangelho, para o legalismo e libert…</t>
-        </is>
-      </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t>Y153</t>
+          <t>P196</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>29/01/2019</t>
+          <t>04/02/2019</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>27/01/2019</t>
+          <t>03/02/2019</t>
         </is>
       </c>
       <c r="C408" t="n">
@@ -35068,7 +35068,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>Série: Síndrome dos Gálatas (parte 2) - Leandro Vieira</t>
+          <t>Série: Síndrome dos Gálatas (parte 3) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E408" t="inlineStr">
@@ -35078,7 +35078,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Gl 3.15-25</t>
+          <t>Gl 1</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -35088,7 +35088,7 @@
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t>Gl 3</t>
+          <t>Gl 1</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
@@ -35113,12 +35113,12 @@
       </c>
       <c r="M408" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=7KUDrbdAhOw</t>
+          <t>https://www.youtube.com/watch?v=qMRyQ6JDeZc</t>
         </is>
       </c>
       <c r="N408" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/sindrome-dos-galatas-parte-02-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/sindrome-dos-galatas-parte-03-leandro-vieira</t>
         </is>
       </c>
       <c r="O408" t="inlineStr">
@@ -35128,34 +35128,29 @@
       </c>
       <c r="P408" t="inlineStr">
         <is>
-          <t>NotebookLM</t>
+          <t>Transcrição do áudio</t>
         </is>
       </c>
       <c r="Q408" t="inlineStr">
         <is>
-          <t>…la para nossa edificação. Então, estamos expondo a Ipislaus Galatas, eu fui até o capítulo 3, hoje eu vou tornar um pouquinho em fatizar um pouco o capítulo 1, mas basicamente qual era o problema acontecendo na igreja da Galáci…</t>
-        </is>
-      </c>
-      <c r="R408" t="inlineStr">
-        <is>
-          <t>Gálatas 3:15-25; Mateus 5:17; Jeremias 31:31-34; 1 Coríntios 2:6-16</t>
+          <t>…m literatura. Amém? Por favor, irmão. Dedique tempo. Vamos agálatas. Capítulo 1. Galatas Capítulo 1, quem encontrou e diga assim. Então, qual é o tema da palavra, as síndromes dos galatas do Evangelho, para o legalismo e libert…</t>
         </is>
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t>Y152</t>
+          <t>Y153</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>23/01/2019</t>
+          <t>29/01/2019</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>20/01/2019</t>
+          <t>27/01/2019</t>
         </is>
       </c>
       <c r="C409" t="n">
@@ -35163,7 +35158,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Introdução à Série: Síndrome dos Gálatas - Leandro Vieira</t>
+          <t>Série: Síndrome dos Gálatas (parte 2) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -35173,7 +35168,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Gl 1.6-9</t>
+          <t>Gl 3.15-25</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -35183,7 +35178,7 @@
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t>Gl 1</t>
+          <t>Gl 3</t>
         </is>
       </c>
       <c r="I409" t="inlineStr">
@@ -35208,44 +35203,49 @@
       </c>
       <c r="M409" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Q-fSPBY7eLI</t>
+          <t>https://www.youtube.com/watch?v=7KUDrbdAhOw</t>
         </is>
       </c>
       <c r="N409" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/sindrome-dos-galatas-leandro-vieira</t>
+          <t>https://soundcloud.com/familiadosquecreem/sindrome-dos-galatas-parte-02-leandro-vieira</t>
         </is>
       </c>
       <c r="O409" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
       <c r="P409" t="inlineStr">
         <is>
-          <t>Transcrição do áudio</t>
+          <t>NotebookLM</t>
         </is>
       </c>
       <c r="Q409" t="inlineStr">
         <is>
-          <t>…e aos irmãos que estavam na Galácia. Então tome sua bíblia, gálatas capítulo 1. Espero terminar hoje essa palavra, senão. Terminamos a próxima semana, mas acredito que eu consigo terminar hoje. Galatas capítulo 1. Hoje nós vamo…</t>
+          <t>…la para nossa edificação. Então, estamos expondo a Ipislaus Galatas, eu fui até o capítulo 3, hoje eu vou tornar um pouquinho em fatizar um pouco o capítulo 1, mas basicamente qual era o problema acontecendo na igreja da Galáci…</t>
+        </is>
+      </c>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t>Gálatas 3:15-25; Mateus 5:17; Jeremias 31:31-34; 1 Coríntios 2:6-16</t>
         </is>
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t>Y151</t>
+          <t>Y152</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>15/01/2019</t>
+          <t>23/01/2019</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>13/01/2019</t>
+          <t>20/01/2019</t>
         </is>
       </c>
       <c r="C410" t="n">
@@ -35253,7 +35253,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>Sacerdócio ao Mundo - Leandro Vieira [Série: Céus | Igreja | Terra]</t>
+          <t>Introdução à Série: Síndrome dos Gálatas - Leandro Vieira</t>
         </is>
       </c>
       <c r="E410" t="inlineStr">
@@ -35263,22 +35263,22 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Nm 20.7-13</t>
+          <t>Gl 1.6-9</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
         <is>
-          <t>Números</t>
+          <t>Gálatas</t>
         </is>
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>Nm 20</t>
+          <t>Gl 1</t>
         </is>
       </c>
       <c r="I410" t="inlineStr">
         <is>
-          <t>Antigo Testamento</t>
+          <t>Novo Testamento</t>
         </is>
       </c>
       <c r="J410" t="inlineStr">
@@ -35288,7 +35288,7 @@
       </c>
       <c r="K410" t="inlineStr">
         <is>
-          <t>Céus | Igreja | Terra</t>
+          <t>Síndrome dos Gálatas</t>
         </is>
       </c>
       <c r="L410" t="inlineStr">
@@ -35298,12 +35298,12 @@
       </c>
       <c r="M410" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=lM3C5cCx-GI</t>
+          <t>https://www.youtube.com/watch?v=Q-fSPBY7eLI</t>
         </is>
       </c>
       <c r="N410" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-sacerdocio-ao-mundo-leandro-vieira-serie-ceus-igreja-terra</t>
+          <t>https://soundcloud.com/familiadosquecreem/sindrome-dos-galatas-leandro-vieira</t>
         </is>
       </c>
       <c r="O410" t="inlineStr">
@@ -35313,29 +35313,29 @@
       </c>
       <c r="P410" t="inlineStr">
         <is>
-          <t>Transcrição + NotebookLM</t>
+          <t>Transcrição do áudio</t>
         </is>
       </c>
       <c r="Q410" t="inlineStr">
         <is>
-          <t>…tendeu? É um projeto por... Quarta para 18 lá, Rosinha. Põe números 18 para... Números 20, 23. Versículo 7, desculpa, Rosa. É que o texto vai até o 23. Falou o Senhor a Moisésia dizendo. Toma a tua vara, ajuda a congregação, tu…</t>
-        </is>
-      </c>
-      <c r="R410" t="inlineStr">
-        <is>
-          <t>Efésios 1:10; Colossenses 1:20; Números 20:7-13; Ezequiel 8:3; Números 16:41-50</t>
+          <t>…e aos irmãos que estavam na Galácia. Então tome sua bíblia, gálatas capítulo 1. Espero terminar hoje essa palavra, senão. Terminamos a próxima semana, mas acredito que eu consigo terminar hoje. Galatas capítulo 1. Hoje nós vamo…</t>
         </is>
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t>Y169</t>
+          <t>Y151</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>~2019 (aprox.)</t>
+          <t>15/01/2019</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>13/01/2019</t>
         </is>
       </c>
       <c r="C411" t="n">
@@ -35343,27 +35343,27 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>O Nosso Resgatador - Leandro Alves</t>
+          <t>Sacerdócio ao Mundo - Leandro Vieira [Série: Céus | Igreja | Terra]</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>Rt 1–4</t>
+          <t>Nm 20.7-13</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
         <is>
-          <t>Rute</t>
+          <t>Números</t>
         </is>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>Rt 1–4</t>
+          <t>Nm 20</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
@@ -35378,7 +35378,7 @@
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t>Fundamentos do NT</t>
+          <t>Céus | Igreja | Terra</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
@@ -35388,27 +35388,37 @@
       </c>
       <c r="M411" s="2" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=jFc2sOuPvys</t>
+          <t>https://www.youtube.com/watch?v=lM3C5cCx-GI</t>
+        </is>
+      </c>
+      <c r="N411" s="2" t="inlineStr">
+        <is>
+          <t>https://soundcloud.com/familiadosquecreem/o-sacerdocio-ao-mundo-leandro-vieira-serie-ceus-igreja-terra</t>
         </is>
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
       <c r="P411" t="inlineStr">
         <is>
-          <t>NotebookLM</t>
+          <t>Transcrição + NotebookLM</t>
+        </is>
+      </c>
+      <c r="Q411" t="inlineStr">
+        <is>
+          <t>…tendeu? É um projeto por... Quarta para 18 lá, Rosinha. Põe números 18 para... Números 20, 23. Versículo 7, desculpa, Rosa. É que o texto vai até o 23. Falou o Senhor a Moisésia dizendo. Toma a tua vara, ajuda a congregação, tu…</t>
         </is>
       </c>
       <c r="R411" t="inlineStr">
         <is>
-          <t>Rute 1:1-21; 2:5-12; 3:9-12; 4:6-18</t>
+          <t>Efésios 1:10; Colossenses 1:20; Números 20:7-13; Ezequiel 8:3; Números 16:41-50</t>
         </is>
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t>Y164</t>
+          <t>Y169</t>
         </is>
       </c>
     </row>
@@ -36788,7 +36798,7 @@
       </c>
       <c r="N428" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-evangelho-completo-part08</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-evangelho-eterno-02</t>
         </is>
       </c>
       <c r="O428" t="inlineStr">
@@ -37283,7 +37293,7 @@
       </c>
       <c r="N434" s="2" t="inlineStr">
         <is>
-          <t>https://soundcloud.com/familiadosquecreem/o-evangelho-da-graca-02</t>
+          <t>https://soundcloud.com/familiadosquecreem/o-evangelho-da-graca-01</t>
         </is>
       </c>
       <c r="O434" t="inlineStr">
@@ -38813,59 +38823,60 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M410" r:id="rId809"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N410" r:id="rId810"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M411" r:id="rId811"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M412" r:id="rId812"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M413" r:id="rId813"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M414" r:id="rId814"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M415" r:id="rId815"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N415" r:id="rId816"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M416" r:id="rId817"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N416" r:id="rId818"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M417" r:id="rId819"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N417" r:id="rId820"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M418" r:id="rId821"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N418" r:id="rId822"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M419" r:id="rId823"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N419" r:id="rId824"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M420" r:id="rId825"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N420" r:id="rId826"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M421" r:id="rId827"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N421" r:id="rId828"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M422" r:id="rId829"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N422" r:id="rId830"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M423" r:id="rId831"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N423" r:id="rId832"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M424" r:id="rId833"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N424" r:id="rId834"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M425" r:id="rId835"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N425" r:id="rId836"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M426" r:id="rId837"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N426" r:id="rId838"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M427" r:id="rId839"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N427" r:id="rId840"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M428" r:id="rId841"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N428" r:id="rId842"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M429" r:id="rId843"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N429" r:id="rId844"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M430" r:id="rId845"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N430" r:id="rId846"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M431" r:id="rId847"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N431" r:id="rId848"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M432" r:id="rId849"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N432" r:id="rId850"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M433" r:id="rId851"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N433" r:id="rId852"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M434" r:id="rId853"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N434" r:id="rId854"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M435" r:id="rId855"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N435" r:id="rId856"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M436" r:id="rId857"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M437" r:id="rId858"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M438" r:id="rId859"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M439" r:id="rId860"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M440" r:id="rId861"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M441" r:id="rId862"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M442" r:id="rId863"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M443" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N411" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M412" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M413" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M414" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M415" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N415" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M416" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N416" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M417" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N417" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M418" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N418" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M419" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N419" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M420" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N420" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M421" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N421" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M422" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N422" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M423" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N423" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M424" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N424" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M425" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N425" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M426" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N426" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M427" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N427" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M428" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N428" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M429" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N429" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M430" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N430" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M431" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N431" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M432" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N432" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M433" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N433" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M434" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N434" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M435" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N435" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M436" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M437" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M438" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M439" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M440" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M441" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M442" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M443" r:id="rId865"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -60975,12 +60986,12 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>P193</t>
+          <t>Y164</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>20/05/2019</t>
+          <t>23/05/2019</t>
         </is>
       </c>
       <c r="C424" t="n">
@@ -60988,27 +60999,32 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Rápidos para Ouvir - Fabiano Krehnke</t>
+          <t>O Nosso Resgatador - Leandro Alves</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>Fabiano Krehnke</t>
+          <t>Leandro Alves</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t>Tiago</t>
+          <t>Rute</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t>Cartas gerais</t>
+          <t>Históricos</t>
         </is>
       </c>
       <c r="J424" t="n">
@@ -61016,19 +61032,19 @@
       </c>
       <c r="K424" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>P194</t>
+          <t>Y164</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>10/05/2019</t>
+          <t>23/05/2019</t>
         </is>
       </c>
       <c r="C425" t="n">
@@ -61036,31 +61052,36 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>O Poder da Ressurreição - Leandro Vieira</t>
+          <t>O Nosso Resgatador - Leandro Alves</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Leandro Alves</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
         <is>
-          <t>2 Tessalonicenses</t>
+          <t>Rute</t>
         </is>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t>Cartas de Paulo</t>
+          <t>Históricos</t>
         </is>
       </c>
       <c r="J425" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K425" t="inlineStr">
         <is>
@@ -61071,12 +61092,12 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>P195</t>
+          <t>Y164</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>06/05/2019</t>
+          <t>23/05/2019</t>
         </is>
       </c>
       <c r="C426" t="n">
@@ -61084,17 +61105,22 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Valor de Uma História Profética - Leandro Vieira</t>
+          <t>O Nosso Resgatador - Leandro Alves</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Leandro Alves</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G426" t="inlineStr">
         <is>
-          <t>Salmos</t>
+          <t>Rute</t>
         </is>
       </c>
       <c r="H426" t="inlineStr">
@@ -61104,11 +61130,11 @@
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t>Poéticos</t>
+          <t>Históricos</t>
         </is>
       </c>
       <c r="J426" t="n">
-        <v>139</v>
+        <v>3</v>
       </c>
       <c r="K426" t="inlineStr">
         <is>
@@ -61119,12 +61145,12 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Y163</t>
+          <t>Y164</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>24/04/2019</t>
+          <t>23/05/2019</t>
         </is>
       </c>
       <c r="C427" t="n">
@@ -61132,7 +61158,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 3) - Leandro Alves</t>
+          <t>O Nosso Resgatador - Leandro Alves</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
@@ -61147,37 +61173,37 @@
       </c>
       <c r="G427" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>Rute</t>
         </is>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t>Evangelhos</t>
+          <t>Históricos</t>
         </is>
       </c>
       <c r="J427" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K427" t="inlineStr">
         <is>
-          <t>Incerto</t>
+          <t>Provável</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>Y162</t>
+          <t>P193</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>03/04/2019</t>
+          <t>20/05/2019</t>
         </is>
       </c>
       <c r="C428" t="n">
@@ -61185,22 +61211,17 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 2) - Felipe Bartoszewski</t>
+          <t>Rápidos para Ouvir - Fabiano Krehnke</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>Felipe Bartoszewski</t>
-        </is>
-      </c>
-      <c r="F428" t="inlineStr">
-        <is>
-          <t>Fundamentos do NT</t>
+          <t>Fabiano Krehnke</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>Tiago</t>
         </is>
       </c>
       <c r="H428" t="inlineStr">
@@ -61210,11 +61231,11 @@
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t>Evangelhos</t>
+          <t>Cartas gerais</t>
         </is>
       </c>
       <c r="J428" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K428" t="inlineStr">
         <is>
@@ -61225,12 +61246,12 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>Y161</t>
+          <t>P194</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>29/03/2019</t>
+          <t>10/05/2019</t>
         </is>
       </c>
       <c r="C429" t="n">
@@ -61238,7 +61259,7 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 1) - Leandro Vieira</t>
+          <t>O Poder da Ressurreição - Leandro Vieira</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
@@ -61246,14 +61267,9 @@
           <t>Leandro Vieira</t>
         </is>
       </c>
-      <c r="F429" t="inlineStr">
-        <is>
-          <t>Fundamentos do NT</t>
-        </is>
-      </c>
       <c r="G429" t="inlineStr">
         <is>
-          <t>Marcos</t>
+          <t>2 Tessalonicenses</t>
         </is>
       </c>
       <c r="H429" t="inlineStr">
@@ -61263,27 +61279,27 @@
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t>Evangelhos</t>
+          <t>Cartas de Paulo</t>
         </is>
       </c>
       <c r="J429" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K429" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Y161</t>
+          <t>P195</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>29/03/2019</t>
+          <t>06/05/2019</t>
         </is>
       </c>
       <c r="C430" t="n">
@@ -61291,7 +61307,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Fundamentos: Reino (parte 1) - Leandro Vieira</t>
+          <t>Valor de Uma História Profética - Leandro Vieira</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
@@ -61299,44 +61315,39 @@
           <t>Leandro Vieira</t>
         </is>
       </c>
-      <c r="F430" t="inlineStr">
-        <is>
-          <t>Fundamentos do NT</t>
-        </is>
-      </c>
       <c r="G430" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Salmos</t>
         </is>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t>Evangelhos</t>
+          <t>Poéticos</t>
         </is>
       </c>
       <c r="J430" t="n">
-        <v>11</v>
+        <v>139</v>
       </c>
       <c r="K430" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Y160</t>
+          <t>Y163</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>22/03/2019</t>
+          <t>24/04/2019</t>
         </is>
       </c>
       <c r="C431" t="n">
@@ -61344,12 +61355,12 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Fundamentos: Cruz (parte 02) - Leandro Vieira</t>
+          <t>Fundamentos: Reino (parte 3) - Leandro Alves</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Leandro Alves</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
@@ -61359,7 +61370,7 @@
       </c>
       <c r="G431" t="inlineStr">
         <is>
-          <t>Gálatas</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H431" t="inlineStr">
@@ -61369,27 +61380,27 @@
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>Cartas de Paulo</t>
+          <t>Evangelhos</t>
         </is>
       </c>
       <c r="J431" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K431" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Incerto</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>Y159</t>
+          <t>Y162</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>18/03/2019</t>
+          <t>03/04/2019</t>
         </is>
       </c>
       <c r="C432" t="n">
@@ -61397,12 +61408,12 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Fundamentos: Cruz (parte 01) - Leandro Vieira</t>
+          <t>Fundamentos: Reino (parte 2) - Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
@@ -61412,7 +61423,7 @@
       </c>
       <c r="G432" t="inlineStr">
         <is>
-          <t>1 Coríntios</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H432" t="inlineStr">
@@ -61422,11 +61433,11 @@
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t>Cartas de Paulo</t>
+          <t>Evangelhos</t>
         </is>
       </c>
       <c r="J432" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K432" t="inlineStr">
         <is>
@@ -61437,12 +61448,12 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>Y158</t>
+          <t>Y161</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>11/03/2019</t>
+          <t>29/03/2019</t>
         </is>
       </c>
       <c r="C433" t="n">
@@ -61450,12 +61461,12 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Fundamentos: Igreja - Leandro Alves</t>
+          <t>Fundamentos: Reino (parte 1) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
@@ -61465,7 +61476,7 @@
       </c>
       <c r="G433" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>Marcos</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">
@@ -61479,7 +61490,7 @@
         </is>
       </c>
       <c r="J433" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K433" t="inlineStr">
         <is>
@@ -61490,12 +61501,12 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>Y157</t>
+          <t>Y161</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>01/03/2019</t>
+          <t>29/03/2019</t>
         </is>
       </c>
       <c r="C434" t="n">
@@ -61503,7 +61514,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Fundamentos: Cristo (parte 02) - Leandro Vieira</t>
+          <t>Fundamentos: Reino (parte 1) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
@@ -61518,7 +61529,7 @@
       </c>
       <c r="G434" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="H434" t="inlineStr">
@@ -61532,7 +61543,7 @@
         </is>
       </c>
       <c r="J434" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="K434" t="inlineStr">
         <is>
@@ -61543,12 +61554,12 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>Y156</t>
+          <t>Y160</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>19/02/2019</t>
+          <t>22/03/2019</t>
         </is>
       </c>
       <c r="C435" t="n">
@@ -61556,12 +61567,12 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Fundamentos: Cristo (parte 01) - Fabiano Krehnke</t>
+          <t>Fundamentos: Cruz (parte 02) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>Fabiano Krehnke</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
@@ -61571,7 +61582,7 @@
       </c>
       <c r="G435" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>Gálatas</t>
         </is>
       </c>
       <c r="H435" t="inlineStr">
@@ -61581,11 +61592,11 @@
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>Evangelhos</t>
+          <t>Cartas de Paulo</t>
         </is>
       </c>
       <c r="J435" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="K435" t="inlineStr">
         <is>
@@ -61596,12 +61607,12 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>Y155</t>
+          <t>Y159</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>16/02/2019</t>
+          <t>18/03/2019</t>
         </is>
       </c>
       <c r="C436" t="n">
@@ -61609,7 +61620,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Introdução aos Fundamentos do NT - Leandro Vieira</t>
+          <t>Fundamentos: Cruz (parte 01) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
@@ -61624,7 +61635,7 @@
       </c>
       <c r="G436" t="inlineStr">
         <is>
-          <t>Mateus</t>
+          <t>1 Coríntios</t>
         </is>
       </c>
       <c r="H436" t="inlineStr">
@@ -61634,11 +61645,11 @@
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>Evangelhos</t>
+          <t>Cartas de Paulo</t>
         </is>
       </c>
       <c r="J436" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="K436" t="inlineStr">
         <is>
@@ -61649,12 +61660,12 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>P196</t>
+          <t>Y158</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>07/02/2019</t>
+          <t>11/03/2019</t>
         </is>
       </c>
       <c r="C437" t="n">
@@ -61662,17 +61673,22 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Batismo nas Águas, no Espírito e no Corpo - Felipe Bartoszewski</t>
+          <t>Fundamentos: Igreja - Leandro Alves</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>Felipe Bartoszewski</t>
+          <t>Leandro Alves</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
         <is>
-          <t>Hebreus</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H437" t="inlineStr">
@@ -61682,27 +61698,27 @@
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>Cartas gerais</t>
+          <t>Evangelhos</t>
         </is>
       </c>
       <c r="J437" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="K437" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>P196</t>
+          <t>Y157</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>07/02/2019</t>
+          <t>01/03/2019</t>
         </is>
       </c>
       <c r="C438" t="n">
@@ -61710,17 +61726,22 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Batismo nas Águas, no Espírito e no Corpo - Felipe Bartoszewski</t>
+          <t>Fundamentos: Cristo (parte 02) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>Felipe Bartoszewski</t>
+          <t>Leandro Vieira</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
         <is>
-          <t>Hebreus</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H438" t="inlineStr">
@@ -61730,27 +61751,27 @@
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>Cartas gerais</t>
+          <t>Evangelhos</t>
         </is>
       </c>
       <c r="J438" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="K438" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>Y153</t>
+          <t>Y156</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>04/02/2019</t>
+          <t>19/02/2019</t>
         </is>
       </c>
       <c r="C439" t="n">
@@ -61758,22 +61779,22 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Série: Síndrome dos Gálatas (parte 3) - Leandro Vieira</t>
+          <t>Fundamentos: Cristo (parte 01) - Fabiano Krehnke</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
+          <t>Fabiano Krehnke</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Síndrome dos Gálatas</t>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G439" t="inlineStr">
         <is>
-          <t>Gálatas</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H439" t="inlineStr">
@@ -61783,27 +61804,27 @@
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t>Cartas de Paulo</t>
+          <t>Evangelhos</t>
         </is>
       </c>
       <c r="J439" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="K439" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>Y152</t>
+          <t>Y155</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>29/01/2019</t>
+          <t>16/02/2019</t>
         </is>
       </c>
       <c r="C440" t="n">
@@ -61811,7 +61832,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Série: Síndrome dos Gálatas (parte 2) - Leandro Vieira</t>
+          <t>Introdução aos Fundamentos do NT - Leandro Vieira</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
@@ -61821,12 +61842,12 @@
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t>Síndrome dos Gálatas</t>
+          <t>Fundamentos do NT</t>
         </is>
       </c>
       <c r="G440" t="inlineStr">
         <is>
-          <t>Gálatas</t>
+          <t>Mateus</t>
         </is>
       </c>
       <c r="H440" t="inlineStr">
@@ -61836,27 +61857,27 @@
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t>Cartas de Paulo</t>
+          <t>Evangelhos</t>
         </is>
       </c>
       <c r="J440" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="K440" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>Y151</t>
+          <t>P196</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>23/01/2019</t>
+          <t>07/02/2019</t>
         </is>
       </c>
       <c r="C441" t="n">
@@ -61864,22 +61885,17 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Introdução à Série: Síndrome dos Gálatas - Leandro Vieira</t>
+          <t>Batismo nas Águas, no Espírito e no Corpo - Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
-        </is>
-      </c>
-      <c r="F441" t="inlineStr">
-        <is>
-          <t>Síndrome dos Gálatas</t>
+          <t>Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
         <is>
-          <t>Gálatas</t>
+          <t>Hebreus</t>
         </is>
       </c>
       <c r="H441" t="inlineStr">
@@ -61889,27 +61905,27 @@
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>Cartas de Paulo</t>
+          <t>Cartas gerais</t>
         </is>
       </c>
       <c r="J441" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>Y169</t>
+          <t>P196</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>15/01/2019</t>
+          <t>07/02/2019</t>
         </is>
       </c>
       <c r="C442" t="n">
@@ -61917,47 +61933,47 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Sacerdócio ao Mundo - Leandro Vieira [Série: Céus | Igreja | Terra]</t>
+          <t>Batismo nas Águas, no Espírito e no Corpo - Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>Leandro Vieira</t>
-        </is>
-      </c>
-      <c r="F442" t="inlineStr">
-        <is>
-          <t>Céus | Igreja | Terra</t>
+          <t>Felipe Bartoszewski</t>
         </is>
       </c>
       <c r="G442" t="inlineStr">
         <is>
-          <t>Números</t>
+          <t>Hebreus</t>
         </is>
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>NT</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t>Pentateuco</t>
+          <t>Cartas gerais</t>
         </is>
       </c>
       <c r="J442" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="K442" t="inlineStr">
         <is>
-          <t>Confirmado</t>
+          <t>Provável</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>Y164</t>
+          <t>Y153</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>04/02/2019</t>
         </is>
       </c>
       <c r="C443" t="n">
@@ -61965,32 +61981,32 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>O Nosso Resgatador - Leandro Alves</t>
+          <t>Série: Síndrome dos Gálatas (parte 3) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Fundamentos do NT</t>
+          <t>Síndrome dos Gálatas</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
         <is>
-          <t>Rute</t>
+          <t>Gálatas</t>
         </is>
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>NT</t>
         </is>
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t>Históricos</t>
+          <t>Cartas de Paulo</t>
         </is>
       </c>
       <c r="J443" t="n">
@@ -62005,7 +62021,12 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>Y164</t>
+          <t>Y152</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>29/01/2019</t>
         </is>
       </c>
       <c r="C444" t="n">
@@ -62013,36 +62034,36 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>O Nosso Resgatador - Leandro Alves</t>
+          <t>Série: Síndrome dos Gálatas (parte 2) - Leandro Vieira</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>Fundamentos do NT</t>
+          <t>Síndrome dos Gálatas</t>
         </is>
       </c>
       <c r="G444" t="inlineStr">
         <is>
-          <t>Rute</t>
+          <t>Gálatas</t>
         </is>
       </c>
       <c r="H444" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>NT</t>
         </is>
       </c>
       <c r="I444" t="inlineStr">
         <is>
-          <t>Históricos</t>
+          <t>Cartas de Paulo</t>
         </is>
       </c>
       <c r="J444" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K444" t="inlineStr">
         <is>
@@ -62053,7 +62074,12 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>Y164</t>
+          <t>Y151</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>23/01/2019</t>
         </is>
       </c>
       <c r="C445" t="n">
@@ -62061,47 +62087,52 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>O Nosso Resgatador - Leandro Alves</t>
+          <t>Introdução à Série: Síndrome dos Gálatas - Leandro Vieira</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>Fundamentos do NT</t>
+          <t>Síndrome dos Gálatas</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
         <is>
-          <t>Rute</t>
+          <t>Gálatas</t>
         </is>
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>NT</t>
         </is>
       </c>
       <c r="I445" t="inlineStr">
         <is>
-          <t>Históricos</t>
+          <t>Cartas de Paulo</t>
         </is>
       </c>
       <c r="J445" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K445" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>Y164</t>
+          <t>Y169</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>15/01/2019</t>
         </is>
       </c>
       <c r="C446" t="n">
@@ -62109,22 +62140,22 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>O Nosso Resgatador - Leandro Alves</t>
+          <t>Sacerdócio ao Mundo - Leandro Vieira [Série: Céus | Igreja | Terra]</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>Leandro Alves</t>
+          <t>Leandro Vieira</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>Fundamentos do NT</t>
+          <t>Céus | Igreja | Terra</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
         <is>
-          <t>Rute</t>
+          <t>Números</t>
         </is>
       </c>
       <c r="H446" t="inlineStr">
@@ -62134,15 +62165,15 @@
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t>Históricos</t>
+          <t>Pentateuco</t>
         </is>
       </c>
       <c r="J446" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="K446" t="inlineStr">
         <is>
-          <t>Provável</t>
+          <t>Confirmado</t>
         </is>
       </c>
     </row>

</xml_diff>